<commit_message>
Actualizar la carta a la versión oficial de Boró
Transcribe carta_boro_cafe_editable_v3.pptx sin cambiar precios ni nombres:
entra el grupo Combos (promos de la mañana y los cuatro combos), los cafés
quedan con su descripción y separados uno por uno, los almuerzos y las
tartaletas dejan de tener precio único, y sale lo que no aparece en la carta
oficial (desayunos, cornetto de jamón queso y los panes chicos).

La dirección pasa a "Los Leones esq Tranquila, Providencia", como en la carta
oficial, en el pie del sitio, la tarjeta de mesa y los metadatos. La navegación
acomoda 3 botones por fila cuando hay más de cuatro grupos.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/carta.xlsx
+++ b/datos/carta.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Carta'!$A$1:$F$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Carta'!$A$1:$F$58</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -83,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -101,6 +101,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -480,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -526,18 +529,18 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Combos</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Calientes</t>
+          <t>Promos de la mañana</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Leche vegetal en cualquier café +$800</t>
+          <t>De lunes a viernes, de 8:00 a 10:30</t>
         </is>
       </c>
       <c r="E2" s="3" t="n"/>
@@ -550,21 +553,26 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Combos</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Calientes</t>
+          <t>Promos de la mañana</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Ristretto / Espresso</t>
+          <t>Café ristretto, espresso, americano o lungo</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Con cualquier compra de salados o dulces</t>
         </is>
       </c>
       <c r="E3" s="4" t="n">
-        <v>3200</v>
+        <v>2500</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -575,21 +583,26 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Combos</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Calientes</t>
+          <t>Promos de la mañana</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Americano / Lungo</t>
+          <t>Café macchiato, cappuccino, latte o flat white</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Con cualquier compra de salados o dulces · Con leche de avena, +$800</t>
         </is>
       </c>
       <c r="E4" s="4" t="n">
-        <v>3300</v>
+        <v>3000</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -598,25 +611,30 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Café</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Calientes</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Machiatto</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>3400</v>
-      </c>
-      <c r="F5" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Combos</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Combos</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Desayuno Liviano</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Café + yogurt con granola</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>4900</v>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -625,21 +643,26 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Combos</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Calientes</t>
+          <t>Combos</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Capuccino</t>
+          <t>Brunch</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Café + jugo de naranja + croissant jamón queso + dulce chico (palmerita, rollo de canela o galleta chocochips)</t>
         </is>
       </c>
       <c r="E6" s="4" t="n">
-        <v>3700</v>
+        <v>10900</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -650,21 +673,26 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Combos</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Calientes</t>
+          <t>Combos</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Latte / Flat white</t>
+          <t>Almuerzo + Bebestible</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Cualquier almuerzo + bebida</t>
         </is>
       </c>
       <c r="E7" s="4" t="n">
-        <v>4000</v>
+        <v>7900</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -675,21 +703,26 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Combos</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Calientes</t>
+          <t>Combos</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Mocaccino / Dirty chai latte</t>
+          <t>Once de Barrio</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Café + dulce chico (palmerita, rollo de canela o galleta chocochips)</t>
         </is>
       </c>
       <c r="E8" s="4" t="n">
-        <v>4500</v>
+        <v>4900</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -698,51 +731,54 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Café</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Calientes</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Chocolate caliente</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>4600</v>
-      </c>
-      <c r="F9" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Café</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Café de especialidad</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Trabajamos grano de especialidad, tostado para Boró Café.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="n"/>
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Café</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Fríos</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Cold brew / Ice latte / Ice capuccino</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="6" t="n">
-        <v>4200</v>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Café</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Café de especialidad</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Espresso</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Corto e intenso, nuestro origen del mes</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F10" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -756,16 +792,21 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Fríos</t>
+          <t>Café de especialidad</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Affogato</t>
+          <t>Ristretto</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>El corazón del espresso</t>
         </is>
       </c>
       <c r="E11" s="4" t="n">
-        <v>4600</v>
+        <v>3200</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -781,16 +822,21 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Fríos</t>
+          <t>Café de especialidad</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Ice tea</t>
+          <t>Americano</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Cuerpo suave, para la sobremesa</t>
         </is>
       </c>
       <c r="E12" s="4" t="n">
-        <v>3500</v>
+        <v>3300</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -806,16 +852,21 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Fríos</t>
+          <t>Café de especialidad</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Ice matcha / Ice chai latte</t>
+          <t>Lungo</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Espresso con más tiempo de extracción</t>
         </is>
       </c>
       <c r="E13" s="4" t="n">
-        <v>4600</v>
+        <v>3300</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -824,24 +875,30 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>Café</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Té e infusiones</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>Todos a $4.200</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="n"/>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Café</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Café de especialidad</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Macchiato</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Espresso «manchado» con espuma</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>3400</v>
+      </c>
+      <c r="F14" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -855,15 +912,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Té e infusiones</t>
+          <t>Café de especialidad</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Té / Infusión</t>
-        </is>
-      </c>
-      <c r="E15" s="9" t="n"/>
+          <t>Cappuccino</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Equilibrio clásico de espresso y leche sedosa</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>3700</v>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -878,15 +942,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Té e infusiones</t>
+          <t>Café de especialidad</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Chai latte</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="n"/>
+          <t>Latte</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Leche texturizada, latte art de la casa</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>4000</v>
+      </c>
       <c r="F16" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -901,15 +972,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Té e infusiones</t>
+          <t>Café de especialidad</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Matcha latte</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="n"/>
+          <t>Flat White</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Espresso con una capa fina y sedosa de leche</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>4000</v>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -924,15 +1002,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Té e infusiones</t>
+          <t>Café de especialidad</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Golden milk</t>
-        </is>
-      </c>
-      <c r="E18" s="9" t="n"/>
+          <t>Mocaccino</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Café y chocolate, una mezcla que abraza</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>4500</v>
+      </c>
       <c r="F18" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -940,30 +1025,30 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>Café</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Jugos y bebidas</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Bebidas en lata</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Coca-Cola normal, light y zero · Fanta zero · Sprite zero</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="n">
-        <v>1800</v>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Café</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Café de especialidad</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Dirty Chai Latte</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Café y chai</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>4500</v>
+      </c>
+      <c r="F19" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -977,16 +1062,21 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Jugos y bebidas</t>
+          <t>Café de especialidad</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Agua con o sin gas</t>
+          <t>Chocolate caliente</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Espeso, de verdad</t>
         </is>
       </c>
       <c r="E20" s="4" t="n">
-        <v>1800</v>
+        <v>4600</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -995,50 +1085,48 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Café</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Jugos y bebidas</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Cerveza sin alcohol</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="n">
-        <v>2200</v>
-      </c>
-      <c r="F21" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Café</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Café de especialidad</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Cámbialo a leche vegetal (avena) +$800</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="n"/>
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Café</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Jugos y bebidas</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Jugo de naranja</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="n">
-        <v>3300</v>
-      </c>
-      <c r="F22" t="inlineStr">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Café</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Café y bebidas frías</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="n"/>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>La tendencia que no se va.</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="n"/>
+      <c r="F22" s="7" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -1052,16 +1140,21 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Jugos y bebidas</t>
+          <t>Café y bebidas frías</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Jugo natural</t>
+          <t>Cold Brew</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>12 horas de extracción en frío</t>
         </is>
       </c>
       <c r="E23" s="4" t="n">
-        <v>3900</v>
+        <v>4200</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1070,30 +1163,30 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>Comida</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Desayunos</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Tostadas con mantequilla de campo</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>Con mermelada casera</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="n">
-        <v>4000</v>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Café</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Café y bebidas frías</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Ice Cappuccino</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Cappuccino cremoso más hielo</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>4200</v>
+      </c>
+      <c r="F24" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -1102,17 +1195,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Comida</t>
+          <t>Café</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Desayunos</t>
+          <t>Café y bebidas frías</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Tostadas con palta</t>
+          <t>Iced Latte</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Latte sobre hielo</t>
         </is>
       </c>
       <c r="E25" s="4" t="n">
@@ -1127,21 +1225,26 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Comida</t>
+          <t>Café</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Desayunos</t>
+          <t>Café y bebidas frías</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Yogurt con granola</t>
+          <t>Affogato</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Helado de vainilla ahogado en espresso</t>
         </is>
       </c>
       <c r="E26" s="4" t="n">
-        <v>3500</v>
+        <v>4600</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1152,21 +1255,26 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Comida</t>
+          <t>Café</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Desayunos</t>
+          <t>Café y bebidas frías</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Sándwich pastrami</t>
+          <t>Ice Matcha / Ice Chai Latte</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Verde vibrante o especiado</t>
         </is>
       </c>
       <c r="E27" s="4" t="n">
-        <v>5000</v>
+        <v>4600</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1175,51 +1283,55 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>Comida</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>Sándwiches y salados</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>Prensado jamón queso</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="n"/>
-      <c r="E28" s="6" t="n">
-        <v>4500</v>
-      </c>
-      <c r="F28" s="5" t="inlineStr">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Café</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Café y bebidas frías</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Ice Tea de la casa</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>3500</v>
+      </c>
+      <c r="F28" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Comida</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Sándwiches y salados</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Cornetto jamón queso</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="n">
-        <v>4500</v>
-      </c>
-      <c r="F29" t="inlineStr">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Café</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Té, matcha e infusiones</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Matcha Latte</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Matcha ceremonial batido</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="n">
+        <v>4200</v>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -1228,21 +1340,26 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Comida</t>
+          <t>Café</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Sándwiches y salados</t>
+          <t>Té, matcha e infusiones</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Croissant jamón queso</t>
+          <t>Chai Latte</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Especias que reconfortan</t>
         </is>
       </c>
       <c r="E30" s="4" t="n">
-        <v>5200</v>
+        <v>4200</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1253,21 +1370,26 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Comida</t>
+          <t>Café</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sándwiches y salados</t>
+          <t>Té, matcha e infusiones</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Croissant salmón y queso crema</t>
+          <t>Golden Milk</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Cúrcuma, jengibre y miel</t>
         </is>
       </c>
       <c r="E31" s="4" t="n">
-        <v>6700</v>
+        <v>4200</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1278,21 +1400,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Comida</t>
+          <t>Café</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Sándwiches y salados</t>
+          <t>Té, matcha e infusiones</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Ciabatta caprese</t>
+          <t>Té e infusiones seleccionadas</t>
         </is>
       </c>
       <c r="E32" s="4" t="n">
-        <v>4200</v>
+        <v>3000</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1301,25 +1423,26 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Comida</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Sándwiches y salados</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Ciabatta pollo mediterráneo</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="n">
-        <v>4700</v>
-      </c>
-      <c r="F33" t="inlineStr">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Café</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Bebidas</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Jugo de naranja exprimido</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="n"/>
+      <c r="E33" s="6" t="n">
+        <v>3900</v>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -1328,21 +1451,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Comida</t>
+          <t>Café</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Sándwiches y salados</t>
+          <t>Bebidas</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Baguette roast beef</t>
+          <t>Jugo natural del día</t>
         </is>
       </c>
       <c r="E34" s="4" t="n">
-        <v>5200</v>
+        <v>3600</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -1351,24 +1474,25 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="7" t="inlineStr">
-        <is>
-          <t>Comida</t>
-        </is>
-      </c>
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t>Almuerzos</t>
-        </is>
-      </c>
-      <c r="C35" s="7" t="n"/>
-      <c r="D35" s="7" t="inlineStr">
-        <is>
-          <t>Todos a $6.990</t>
-        </is>
-      </c>
-      <c r="E35" s="8" t="n"/>
-      <c r="F35" s="7" t="inlineStr">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Café</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Bebidas</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Latas de bebida / Agua</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F35" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -1377,54 +1501,49 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>Café</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Bebidas</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Cerveza sin alcohol</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>2200</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
           <t>Comida</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Almuerzos</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Ensaladas</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>César · Quinoa pollo · Salmón ahumado · Vegetariana</t>
-        </is>
-      </c>
-      <c r="E36" s="9" t="n"/>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Comida</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Almuerzos</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Gohans</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Camarón · Pollo teriyaki · Salmón</t>
-        </is>
-      </c>
-      <c r="E37" s="9" t="n"/>
-      <c r="F37" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Salados y sándwiches</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Croissant de jamón y queso</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="n"/>
+      <c r="E37" s="6" t="n">
+        <v>4800</v>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -1438,20 +1557,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Almuerzos</t>
+          <t>Salados y sándwiches</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Pastas</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Fetuccine boloñesa · Lasaña</t>
-        </is>
-      </c>
-      <c r="E38" s="9" t="n"/>
+          <t>Croissant de salmón y queso crema</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>6700</v>
+      </c>
       <c r="F38" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -1466,15 +1582,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Almuerzos</t>
+          <t>Salados y sándwiches</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Wrap</t>
-        </is>
-      </c>
-      <c r="E39" s="9" t="n"/>
+          <t>Baguette de roast beef</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="n">
+        <v>5200</v>
+      </c>
       <c r="F39" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -1482,26 +1600,25 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="inlineStr">
-        <is>
-          <t>Dulces</t>
-        </is>
-      </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>Masas y medialunas</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>Palmerita / Cornetto tradicional</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="n"/>
-      <c r="E40" s="6" t="n">
-        <v>2000</v>
-      </c>
-      <c r="F40" s="5" t="inlineStr">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Salados y sándwiches</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Ciabatta de pollo mediterráneo</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="n">
+        <v>4700</v>
+      </c>
+      <c r="F40" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -1510,21 +1627,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Dulces</t>
+          <t>Comida</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Masas y medialunas</t>
+          <t>Salados y sándwiches</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Rollo de canela</t>
+          <t>Ciabatta Caprese</t>
         </is>
       </c>
       <c r="E41" s="4" t="n">
-        <v>2200</v>
+        <v>4200</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -1535,21 +1652,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Dulces</t>
+          <t>Comida</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Masas y medialunas</t>
+          <t>Salados y sándwiches</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Pan de chocolate</t>
+          <t>Prensado de jamón y queso</t>
         </is>
       </c>
       <c r="E42" s="4" t="n">
-        <v>3600</v>
+        <v>4500</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -1558,51 +1675,58 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Dulces</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Masas y medialunas</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Cornetto Nutella / Pistacho / Pastelera italiana</t>
-        </is>
-      </c>
-      <c r="E43" s="4" t="n">
-        <v>5300</v>
-      </c>
-      <c r="F43" t="inlineStr">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Almuerzos</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Ensaladas</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="n"/>
+      <c r="E43" s="9" t="inlineStr">
+        <is>
+          <t>César · Vegetariana: 6590 / Pollo con quinoa · Salmón ahumado: 6990</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t>Dulces</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="inlineStr">
-        <is>
-          <t>Pastelería</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>Galleta chocochips</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="n"/>
-      <c r="E44" s="6" t="n">
-        <v>2900</v>
-      </c>
-      <c r="F44" s="5" t="inlineStr">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Almuerzos</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Gohans</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Camarón · Pollo teriyaki · Salmón ahumado</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="n">
+        <v>6990</v>
+      </c>
+      <c r="F44" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -1611,21 +1735,26 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Dulces</t>
+          <t>Comida</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Pastelería</t>
+          <t>Almuerzos</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Brookie / Brownie de chocolate</t>
+          <t>Pastas</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Fetuccine boloñesa · Lasaña</t>
         </is>
       </c>
       <c r="E45" s="4" t="n">
-        <v>3400</v>
+        <v>6990</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -1636,53 +1765,51 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>Comida</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Almuerzos</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Wrap del día</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="n">
+        <v>6390</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
           <t>Dulces</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Pastelería</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Tartaletas</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Cheesecake frambuesa · Chocolate menta · Key lime pie</t>
-        </is>
-      </c>
-      <c r="E46" s="4" t="n">
-        <v>3200</v>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Dulces</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Pastelería</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Tartaleta de pistacho</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="n">
-        <v>4200</v>
-      </c>
-      <c r="F47" t="inlineStr">
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Pastelería y dulces</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>Cornetto relleno</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="n"/>
+      <c r="E47" s="9" t="inlineStr">
+        <is>
+          <t>Pastelera italiana: 3700 / Nutella · Pistacho: 4800</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -1696,17 +1823,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Pastelería</t>
+          <t>Pastelería y dulces</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Helados</t>
-        </is>
-      </c>
-      <c r="E48" s="9" t="inlineStr">
-        <is>
-          <t>180 ml: 4500 / 500 ml: 9500</t>
+          <t>Tartaletas</t>
+        </is>
+      </c>
+      <c r="E48" s="10" t="inlineStr">
+        <is>
+          <t>Chocolate menta · Pie de limón: 3400 / Pistacho: 4200</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -1716,24 +1843,25 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="inlineStr">
-        <is>
-          <t>Pan</t>
-        </is>
-      </c>
-      <c r="B49" s="7" t="inlineStr">
-        <is>
-          <t>Pan</t>
-        </is>
-      </c>
-      <c r="C49" s="7" t="n"/>
-      <c r="D49" s="7" t="inlineStr">
-        <is>
-          <t>Para llevar a casa.</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="n"/>
-      <c r="F49" s="7" t="inlineStr">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Dulces</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Pastelería y dulces</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Brookie / Brownie</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="n">
+        <v>3400</v>
+      </c>
+      <c r="F49" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -1742,21 +1870,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Pan</t>
+          <t>Dulces</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Pan</t>
+          <t>Pastelería y dulces</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Pan ciabatta</t>
+          <t>Pan de chocolate</t>
         </is>
       </c>
       <c r="E50" s="4" t="n">
-        <v>990</v>
+        <v>3900</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -1767,21 +1895,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Pan</t>
+          <t>Dulces</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Pan</t>
+          <t>Pastelería y dulces</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Brioche / Mini baguette</t>
+          <t>Galleta chocochips</t>
         </is>
       </c>
       <c r="E51" s="4" t="n">
-        <v>1100</v>
+        <v>2900</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -1792,21 +1920,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Pan</t>
+          <t>Dulces</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Pan</t>
+          <t>Pastelería y dulces</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Baguette de masa madre</t>
+          <t>Rollo de canela</t>
         </is>
       </c>
       <c r="E52" s="4" t="n">
-        <v>2200</v>
+        <v>2400</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -1817,21 +1945,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Pan</t>
+          <t>Dulces</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Pan</t>
+          <t>Pastelería y dulces</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Hogaza 100% integral</t>
+          <t>Palmerita</t>
         </is>
       </c>
       <c r="E53" s="4" t="n">
-        <v>4900</v>
+        <v>2400</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -1842,61 +1970,137 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t>Dulces</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Pastelería y dulces</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Helados artesanales</t>
+        </is>
+      </c>
+      <c r="E54" s="10" t="inlineStr">
+        <is>
+          <t>180 ml: 4500 / 500 ml: 9500</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="7" t="inlineStr">
+        <is>
           <t>Pan</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B55" s="7" t="inlineStr">
         <is>
           <t>Pan</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C55" s="7" t="n"/>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>Para llevar</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="n"/>
+      <c r="F55" s="7" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Pan</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Pan</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
         <is>
           <t>Hogaza blanca de masa madre</t>
         </is>
       </c>
-      <c r="E54" s="4" t="n">
+      <c r="E56" s="4" t="n">
         <v>4800</v>
       </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
         <is>
           <t>Pan</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>Pan</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>Hogaza semi integral de masa madre</t>
         </is>
       </c>
-      <c r="E55" s="4" t="n">
+      <c r="E57" s="4" t="n">
         <v>4900</v>
       </c>
-      <c r="F55" t="inlineStr">
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Pan</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Pan</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Hogaza 100% integral</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="n">
+        <v>4900</v>
+      </c>
+      <c r="F58" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F55"/>
+  <autoFilter ref="A1:F58"/>
   <dataValidations count="2">
-    <dataValidation sqref="F2:F355" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Mostrar" error="Escribe Sí o No." type="list">
+    <dataValidation sqref="F2:F358" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Mostrar" error="Escribe Sí o No." type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="A2:A355" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Grupo nuevo" error="Ese grupo todavía no existe: la carta va a mostrar un botón nuevo." type="list" errorStyle="information">
-      <formula1>"Café,Comida,Dulces,Pan"</formula1>
+    <dataValidation sqref="A2:A358" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Grupo nuevo" error="Ese grupo todavía no existe: la carta va a mostrar un botón nuevo." type="list" errorStyle="information">
+      <formula1>"Combos,Café,Comida,Dulces,Pan"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1916,121 +2120,121 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Carta de Boró Café: cómo actualizarla</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr"/>
+      <c r="A2" s="12" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>EDITAR (hoja «Carta»)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>• Cambiar un precio: escribe el número nuevo en Precio. Solo el número, por ejemplo 3700.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>• Agregar un producto: inserta una fila dentro de su sección y completa Producto y Precio. Si dejas Grupo y Sección vacíos, se usan los de la fila de arriba.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>• Sacar un producto por un tiempo (agotado, de temporada): pon No en Mostrar. Para que vuelva, Sí.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>• Detalle (opcional): texto chico bajo el nombre, por ejemplo «César · Quinoa pollo · Vegetariana».</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>• Productos con tamaños: en Precio escribe «180 ml: 4500 / 500 ml: 9500».</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>• Notas de sección (filas grises): van SIN Producto, con el texto en Detalle. Si la nota empieza con «Todos a» (por ejemplo «Todos a $6.990»), se muestra como sello y los productos de esa sección van sin precio.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>• La carta respeta el orden de las filas. Para una sección o un grupo nuevo, escribe un nombre nuevo: cada grupo es un botón arriba de la carta.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr"/>
+      <c r="A11" s="12" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>PUBLICAR</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>1. Guarda el archivo (sirve Excel, Numbers o Google Sheets descargado como .xlsx o .csv).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>2. Entra a https://github.com/borocafe/carta/upload/main/datos</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>3. Arrastra el archivo (puede tener cualquier nombre) y aprieta «Commit changes».</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>4. En unos 2 minutos la carta está actualizada: https://borocafe.github.io/carta/</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="inlineStr"/>
+      <c r="A17" s="12" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>Si algo está mal escrito, la carta NO cambia y GitHub avisa por correo qué fila revisar. Corrígela y vuelve a subir el archivo.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="inlineStr">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>Para editar siempre la versión más reciente, descárgala de: https://github.com/borocafe/carta/raw/main/datos/carta.xlsx</t>
         </is>

</xml_diff>

<commit_message>
Agrupar como la carta oficial, sacar las ilustraciones y arreglar el sello
Las agrupaciones pasan a ser las de la PPT: Combos, Café & bebidas (de la
barra) y Para comer (de la vitrina). Salen las bandas ilustradas de entre las
secciones; quedan guardadas en marca/anteriores/.

El logo original llega con el anillo cortado en los cuatro bordes:
herramientas/logo.py detecta el círculo real, lo completa y deja margen. De ahí
salen el sello de la portada, el del pie y el del QR.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/carta.xlsx
+++ b/datos/carta.xlsx
@@ -733,7 +733,7 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -757,7 +757,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -787,7 +787,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -817,7 +817,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -847,7 +847,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -877,7 +877,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -907,7 +907,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -937,7 +937,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -967,7 +967,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -997,7 +997,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1027,7 +1027,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1057,7 +1057,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1087,7 +1087,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1111,7 +1111,7 @@
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -1135,7 +1135,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1165,7 +1165,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1195,7 +1195,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1225,7 +1225,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1255,7 +1255,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1285,7 +1285,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1310,7 +1310,7 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -1340,7 +1340,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1400,7 +1400,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1425,7 +1425,7 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
@@ -1451,7 +1451,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1476,7 +1476,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1501,7 +1501,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Café</t>
+          <t>Café &amp; bebidas</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1526,7 +1526,7 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>Comida</t>
+          <t>Para comer</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
@@ -1552,7 +1552,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Comida</t>
+          <t>Para comer</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Comida</t>
+          <t>Para comer</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1602,7 +1602,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Comida</t>
+          <t>Para comer</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1627,7 +1627,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Comida</t>
+          <t>Para comer</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1652,7 +1652,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Comida</t>
+          <t>Para comer</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1677,7 +1677,7 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>Comida</t>
+          <t>Para comer</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
@@ -1705,7 +1705,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Comida</t>
+          <t>Para comer</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1735,7 +1735,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Comida</t>
+          <t>Para comer</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1765,7 +1765,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Comida</t>
+          <t>Para comer</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1790,7 +1790,7 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Dulces</t>
+          <t>Para comer</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
@@ -1818,7 +1818,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Dulces</t>
+          <t>Para comer</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1845,7 +1845,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Dulces</t>
+          <t>Para comer</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1870,7 +1870,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Dulces</t>
+          <t>Para comer</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1895,7 +1895,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Dulces</t>
+          <t>Para comer</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1920,7 +1920,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Dulces</t>
+          <t>Para comer</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1945,7 +1945,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Dulces</t>
+          <t>Para comer</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1970,7 +1970,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Dulces</t>
+          <t>Para comer</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1997,12 +1997,12 @@
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>Pan</t>
+          <t>Para comer</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>Pan</t>
+          <t>Panadería de masa madre</t>
         </is>
       </c>
       <c r="C55" s="7" t="n"/>
@@ -2021,12 +2021,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Pan</t>
+          <t>Para comer</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Pan</t>
+          <t>Panadería de masa madre</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2046,12 +2046,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Pan</t>
+          <t>Para comer</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Pan</t>
+          <t>Panadería de masa madre</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2071,12 +2071,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Pan</t>
+          <t>Para comer</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Pan</t>
+          <t>Panadería de masa madre</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2100,7 +2100,7 @@
       <formula1>"Sí,No"</formula1>
     </dataValidation>
     <dataValidation sqref="A2:A358" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Grupo nuevo" error="Ese grupo todavía no existe: la carta va a mostrar un botón nuevo." type="list" errorStyle="information">
-      <formula1>"Combos,Café,Comida,Dulces,Pan"</formula1>
+      <formula1>"Combos,Café &amp; bebidas,Para comer"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mostrar las promos de la mañana como en la portada de la carta
Las dos promos dejan de ser una lista de precios y pasan a bloques
destacados, con el nombre, el precio y la condición debajo. La regla queda
en la planilla: una sección cuyo nombre empieza con «Promo» se muestra así.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/carta.xlsx
+++ b/datos/carta.xlsx
@@ -563,12 +563,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Café ristretto, espresso, americano o lungo</t>
+          <t>Tu café</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Con cualquier compra de salados o dulces</t>
+          <t>Con cualquier compra de salados o dulces, pide un café ristretto, espresso, americano o lungo.</t>
         </is>
       </c>
       <c r="E3" s="4" t="n">
@@ -593,12 +593,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Café macchiato, cappuccino, latte o flat white</t>
+          <t>Tu café con leche</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Con cualquier compra de salados o dulces · Con leche de avena, +$800</t>
+          <t>Con cualquier compra de salados o dulces, pide tu café macchiato, cappuccino, latte o flat white. Con leche de avena, +$800.</t>
         </is>
       </c>
       <c r="E4" s="4" t="n">
@@ -2113,7 +2113,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -2186,55 +2186,62 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr"/>
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>• Promociones: si el nombre de la sección empieza con «Promo», sus productos se muestran destacados, en recuadros, en vez de la lista de precios normal. Sirve para las promos de la mañana.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>PUBLICAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>1. Guarda el archivo (sirve Excel, Numbers o Google Sheets descargado como .xlsx o .csv).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>2. Entra a https://github.com/borocafe/carta/upload/main/datos</t>
+          <t>1. Guarda el archivo (sirve Excel, Numbers o Google Sheets descargado como .xlsx o .csv).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>3. Arrastra el archivo (puede tener cualquier nombre) y aprieta «Commit changes».</t>
+          <t>2. Entra a https://github.com/borocafe/carta/upload/main/datos</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
+          <t>3. Arrastra el archivo (puede tener cualquier nombre) y aprieta «Commit changes».</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
           <t>4. En unos 2 minutos la carta está actualizada: https://borocafe.github.io/carta/</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="12" t="inlineStr"/>
-    </row>
     <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>Si algo está mal escrito, la carta NO cambia y GitHub avisa por correo qué fila revisar. Corrígela y vuelve a subir el archivo.</t>
-        </is>
-      </c>
+      <c r="A18" s="12" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>Si algo está mal escrito, la carta NO cambia y GitHub avisa por correo qué fila revisar. Corrígela y vuelve a subir el archivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t>Para editar siempre la versión más reciente, descárgala de: https://github.com/borocafe/carta/raw/main/datos/carta.xlsx</t>
         </is>

</xml_diff>